<commit_message>
Settings and Administrator tests added
</commit_message>
<xml_diff>
--- a/downloads/Fleet_Summary.xlsx.xlsx
+++ b/downloads/Fleet_Summary.xlsx.xlsx
@@ -471,19 +471,19 @@
         <v>GCBL10536MHG14AG04459</v>
       </c>
       <c r="C4">
-        <v>39.62</v>
+        <v>0</v>
       </c>
       <c r="D4" t="str">
-        <v>24m</v>
+        <v>1d 14h 20m</v>
       </c>
       <c r="E4" t="str">
-        <v>19h 5m</v>
+        <v>21h 6m</v>
       </c>
       <c r="F4" t="str">
-        <v>24m</v>
+        <v>1d 14h 20m</v>
       </c>
       <c r="G4">
-        <v>35.19</v>
+        <v>0</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -495,7 +495,7 @@
         <v>100</v>
       </c>
       <c r="K4" t="str">
-        <v>2026-09-01 19:05:43</v>
+        <v>2026-09-03 21:06:15</v>
       </c>
       <c r="L4" t="str">
         <v>A</v>
@@ -507,19 +507,19 @@
         <v>Closed</v>
       </c>
       <c r="O4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P4" t="str">
         <v>Mumbai</v>
       </c>
       <c r="Q4">
-        <v>63070.41</v>
+        <v>63086.6</v>
       </c>
       <c r="R4" t="str">
         <v>Sibrampur, West Bengal, India</v>
       </c>
       <c r="S4">
-        <v>5.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>